<commit_message>
Remove source column, source note and source heading from buyers sheet
- drop 'Source (directory record)' column
- drop the bottom note paragraph and the source mention in the title
- replace 'Import Evidence' / 'Notes & Method' with a clean 'Buyer Details' sheet
- validation now fails if any cell or link mentions a source

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/US_Buyers_Lanterns_and_Jewellery.xlsx
+++ b/US_Buyers_Lanterns_and_Jewellery.xlsx
@@ -8,14 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="US Buyers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Import Evidence" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes &amp; Method" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Buyer Details" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'US Buyers'!$A$4:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'US Buyers'!$A$4:$G$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'US Buyers'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Import Evidence'!$A$4:$J$14</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Import Evidence'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Buyer Details'!$A$4:$I$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Buyer Details'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,23 +58,6 @@
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00305496"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -122,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,20 +132,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -530,30 +498,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>US Buyers - Lanterns &amp; Jewellery (source: usa.importers-directory.net)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="26" customHeight="1">
+          <t>US Buyers - Lanterns &amp; Jewellery</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared: 22 October 2026  |  10 buyers: 5 Lanterns, 5 Jewellery  |  Buyer records taken from US Customs bill-of-lading entries on usa.importers-directory.net</t>
+          <t>Prepared: 22 October 2026  |  10 buyers: 5 Lanterns, 5 Jewellery</t>
         </is>
       </c>
     </row>
@@ -594,11 +561,6 @@
           <t>Contact (Phone / E-mail)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Source (directory record)</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -611,7 +573,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Buying Desk - Seasonal &amp; Home (no category buyer named publicly)</t>
+          <t>Buying Desk - Seasonal &amp; Home</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -632,11 +594,6 @@
       <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Vendor submissions via Costco Supplier/Vendor Inquiry on costco.com</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
         </is>
       </c>
     </row>
@@ -651,7 +608,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Buying Desk - Home &amp; Seasonal Decor (no category buyer named publicly)</t>
+          <t>Buying Desk - Home &amp; Seasonal Decor</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -672,11 +629,6 @@
       <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Vendor/partner enquiries via fredmeyer.com; buying office Portland, OR</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
         </is>
       </c>
     </row>
@@ -714,11 +666,6 @@
           <t>Product development &amp; merchandising desk via pier1.com</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="49" customHeight="1">
       <c r="A8" s="7" t="n">
@@ -754,11 +701,6 @@
           <t>contact@styleasia.net | +1 (201) 460-9611 | toll-free (800) 522-7465</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -771,7 +713,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Buying Desk - Hardlines / General Merchandise (no buyer named publicly)</t>
+          <t>Buying Desk - Hardlines / General Merchandise</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -794,13 +736,8 @@
           <t>Vendor enquiries via kmart.com</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/import_data/lantern-1001653566.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="49" customHeight="1">
+    </row>
+    <row r="10" ht="34" customHeight="1">
       <c r="A10" s="7" t="n">
         <v>6</v>
       </c>
@@ -811,7 +748,7 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Buying Desk - Fashion Jewellery &amp; Accessories (no category buyer named publicly)</t>
+          <t>Buying Desk - Fashion Jewellery &amp; Accessories</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -831,16 +768,11 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Merchandising via avon.com; corporate office 165 Broadway, New York, NY 10006</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/jewelry-1001656961.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="49" customHeight="1">
+          <t>Merchandising via avon.com; office 165 Broadway, New York, NY 10006</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
@@ -874,13 +806,8 @@
           <t>scott@barryowen.com | orders@barryowen.com | +1 (323) 724-4800</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/jewelry-1001656961.html ; https://usa.importers-directory.net/bracelet-1007248.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
+    </row>
+    <row r="12" ht="19" customHeight="1">
       <c r="A12" s="7" t="n">
         <v>8</v>
       </c>
@@ -912,11 +839,6 @@
       <c r="G12" s="8" t="inlineStr">
         <is>
           <t>sales@tossdesigns.com | +1 (415) 721-1037</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/jewelry-1001656961.html</t>
         </is>
       </c>
     </row>
@@ -931,7 +853,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Buying Desk - Jewellery &amp; Accessories (no category buyer named publicly)</t>
+          <t>Buying Desk - Jewellery &amp; Accessories</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -954,13 +876,8 @@
           <t>Supplier onboarding via Dollar General supplier portal / vendor enquiry</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/necklace-10071.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
+    </row>
+    <row r="14" ht="19" customHeight="1">
       <c r="A14" s="7" t="n">
         <v>10</v>
       </c>
@@ -971,7 +888,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Import Desk - wholesale showroom (no individual buyer named publicly)</t>
+          <t>Import Desk - wholesale showroom</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -994,25 +911,12 @@
           <t>1261 Broadway, Suite 701, New York, NY 10001</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/necklace-10071.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>All 10 companies appear on usa.importers-directory.net as the 'US Importer' of a lantern or jewellery bill-of-lading entry (see 'Import Evidence'). Freight forwarders and non-US consignees were filtered out. 'Buyer Name' is a named decision-maker only where a public source documents one; otherwise route through the buying desk listed.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H14"/>
-  <mergeCells count="3">
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+  <autoFilter ref="A4:G14"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
@@ -1036,32 +940,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Import Evidence - the directory (B/L) record behind every buyer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="26" customHeight="1">
+          <t>Buyer details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Address columns are exactly as printed in the directory record; 'Current address' updates are in the Notes sheet.</t>
+          <t>Address, product and fit for each buyer.</t>
         </is>
       </c>
     </row>
@@ -1074,51 +977,46 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Company (US Importer on record)</t>
+          <t>Company Name</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Product Category</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Address as printed in directory</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Product description as filed (B/L)</t>
+          <t>Product Imported</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Export port</t>
+          <t>Origin / Export</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>US port</t>
+          <t>US Port of Entry</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Product fit</t>
+          <t>Product Fit</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Current status</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Directory page</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="49" customHeight="1">
+          <t>Current Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -1139,12 +1037,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Large Solar Base Lantern, P.O. 175-0731-260 (803 cartons; shipper Matador International Inc., Taiwan)</t>
+          <t>Large solar base lantern (803 cartons)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Yantian, China</t>
+          <t>China - Yantian</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1154,17 +1052,12 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Medium - solar/garden decor lanterns</t>
+          <t>Medium - solar / garden decor lanterns</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Active - membership warehouse club; new vendors via Costco vendor programme</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1087,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Busan, South Korea</t>
+          <t>South Korea - Busan</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1212,13 +1105,8 @@
           <t>Active - Kroger banner, ~130 stores in the Pacific Northwest</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="49" customHeight="1">
+    </row>
+    <row r="7" ht="34" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
@@ -1234,12 +1122,12 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>609 Kirk Rd, St Charles, IL 60174 (HQ: 100 Pier 1 Place, Fort Worth, TX 76102)</t>
+          <t>100 Pier 1 Place, Fort Worth, TX 76102</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>44 ctns Metal Lantern (shipment also carried glass candle holders, stone plates, paper flowers)</t>
+          <t>Metal lanterns (44 cartons), with candle holders and other decor</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -1260,11 +1148,6 @@
       <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Active - online-only since 2020; sourcing led by Omni Retail Enterprises</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1167,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>210 Moonachie Avenue, Moonachie, NJ 07074 (current: 101 Moonachie Ave)</t>
+          <t>101 Moonachie Avenue, Moonachie, NJ 07074</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -1294,12 +1177,12 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Ningbo, China</t>
+          <t>China - Ningbo</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Not stated on record</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -1310,11 +1193,6 @@
       <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Active - importer &amp; wholesale distributor since 1985 (best-fit wholesale lead)</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/lantern-1001653566.html</t>
         </is>
       </c>
     </row>
@@ -1344,27 +1222,22 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Not stated on record</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Not stated on record</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Low-Medium - utility/camping lanterns rather than decorative</t>
+          <t>Low-Medium - utility / camping lanterns rather than decorative</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Limited - few stores remain under Transformco; kmart.com still trading</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/import_data/lantern-1001653566.html</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1257,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>1251 Avenue of the Americas, New York, NY 10020</t>
+          <t>165 Broadway, New York, NY 10006</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -1412,13 +1285,8 @@
           <t>Active - US business operates as The Avon Company</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/jewelry-1001656961.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="64" customHeight="1">
+    </row>
+    <row r="11" ht="49" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
@@ -1439,12 +1307,12 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Imitation jewelry (lead &amp; nickel free); dolphin/whale-tail pendant bracelets</t>
+          <t>Imitation jewelry (lead &amp; nickel free); pendant bracelets</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Busan, South Korea / Yantian, China</t>
+          <t>South Korea - Busan / China - Yantian</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1460,11 +1328,6 @@
       <c r="I11" s="5" t="inlineStr">
         <is>
           <t>Active - fresh imitation-jewellery imports recorded in 2026</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/jewelry-1001656961.html ; https://usa.importers-directory.net/bracelet-1007248.html</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1347,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>3070 Kerner Blvd, Unit C, San Rafael, CA 94901 (HQ: 343 San Anselmo Ave, San Anselmo, CA 94960)</t>
+          <t>343 San Anselmo Ave, San Anselmo, CA 94960</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1510,11 +1373,6 @@
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Active - design house, wholesaler and own retail stores</t>
-        </is>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/jewelry-1001656961.html</t>
         </is>
       </c>
     </row>
@@ -1539,12 +1397,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Fairy 'N Jewel necklace, P.O. IN2RNX</t>
+          <t>'Fairy N Jewel' necklace</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Yantian, China</t>
+          <t>China - Yantian</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1560,11 +1418,6 @@
       <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Active - ~20,000 stores; central buying from Goodlettsville</t>
-        </is>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/necklace-10071.html</t>
         </is>
       </c>
     </row>
@@ -1584,17 +1437,17 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>22 W 32nd St, 2nd Floor, New York, NY 10001 (current: 1261 Broadway, Suite 701)</t>
+          <t>1261 Broadway, Suite 701, New York, NY 10001</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Bangle &amp; earring &amp; choker necklace &amp; earring &amp; tie</t>
+          <t>Bangles, earrings, choker necklace and tie sets</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Shanghai, China</t>
+          <t>China - Shanghai</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1612,204 +1465,14 @@
           <t>Active - jewellery-set imports recorded through 2026</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>https://usa.importers-directory.net/necklace-10071.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Named-contact sources (checked 22 Oct 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Pier 1 Imports (Omni Retail Enterprises): https://www.businesswire.com/news/home/20241024431906/en/ (Omni names Cindy Kretzinger to lead Pier 1 product development &amp; merchandising)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Style Asia Inc.: https://www.bbb.org/us/nj/moonachie/profile/exporter/style-asia-inc-0221-10002213 (Ashok Pamani, President) ; https://styleasia.net/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>Barry-Owen Co., Inc.: https://www.dnb.com/business-directory/company-profiles.barry-owen_co_inc.fd2b7c0579f5e267efa8bb2855a1a629.html (Scott Fink, President) ; https://barryowen.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>Toss Designs: https://www.dnb.com/business-directory/company-profiles.toss_designs_inc.9bf965cc249886eb9c0b909652696243.html (Jennifer Hogan, key principal) ; https://www.tossdesigns.com/pages/contact-us</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J14"/>
-  <mergeCells count="7">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A18:J18"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="A19:J19"/>
+  <autoFilter ref="A4:I14"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId10"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Notes, method and caveats</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Read this before using the list for outreach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1"/>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>How this list was built</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="75" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>1. Product pages were pulled from usa.importers-directory.net: Lantern (https://usa.importers-directory.net/lantern-1001653566.html), its Buyers page (https://usa.importers-directory.net/buyer/lantern-1001653566.html) and Import-Data page (https://usa.importers-directory.net/import_data/lantern-1001653566.html); Jewellery (https://usa.importers-directory.net/jewelry-1001656961.html), Bracelet (https://usa.importers-directory.net/bracelet-1007248.html) and Necklace (https://usa.importers-directory.net/necklace-10071.html).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>2. Every company on the directory pages that appears as 'US Importer' was reviewed. Freight forwarders, NVOCCs, customs brokers and non-US consignees were removed (e.g. Panalpina, Pan Star Express, Freight Savers, Geologistics, Allied Transport System, Galaxy Freight, Perfect Express, Deltamax, Home Hardware Stores Ltd (Canada)).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>3. The remaining 10 real buyers (5 lanterns, 5 jewellery) were enriched with the current website, address and - where publicly documented - a named decision-maker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>Caveats</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>- Directory records are US Customs bill-of-lading filings. They are historic: they prove the company does buy this product, but the shipment shown may not be recent. Always re-verify before outreach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>- 'Buyer Name' is a named head/decision-maker only where a public source documents it (Pier 1, Style Asia, Barry-Owen, Toss Designs). Category buyers at large retailers (Costco, Fred Meyer, Kmart, Avon, Dollar General) are not published; those rows give the buying desk you must route through instead of inventing a name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>- Eastern Nationwide Supply has no public website; it is a trade-only showroom in the New York jewellery district and can be approached by post/phone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Suggested outreach order</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="75" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>1) Style Asia Inc. - direct importer/distributor, named president &amp; imports manager. 2) Barry-Owen Co. - costume-jewellery importer, named president, actively importing in 2026. 3) Eastern Nationwide Supply - pure-play fashion-jewellery importer. 4) Toss Designs - smaller, design-led, fast decisions. 5) Pier 1 - high fit for decorative metal lanterns, sourcing team in place. 6) Large retailers (Costco, Fred Meyer, Dollar General, Avon, Kmart) - long vendor-onboarding cycles; approach with a factory audit pack, test-report compliance (CPSIA/prop 65) and FOB quotes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Verification dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Directory records pulled: 22 Oct 2026. Website / contact / status checks: 22 Oct 2026. Named-contact sources are on the 'Import Evidence' sheet.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A12:B12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh buyers sheet with 23 Oct 2026 data (5 lanterns + 5 jewellery)
Lanterns: World Market, Lowe's (L G Sourcing), Family Dollar,
Globe Lighting (A-Boy Supply), Pier 1 Imports.
Jewellery: DM Merchandising, Barry-Owen, Toss Designs,
Big Lots (Variety Wholesalers), 5 And 2 Co.

- new records pulled from US Customs importer pages (lantern, candle,
  candle holder, christmas light, lamp, jewelry, necklace, bracelet)
- websites, phones, e-mails and 2026 ownership/status re-verified
- named decision-makers where public: Pat Dolan, Cindy Kretzinger,
  Gavin Marks, Scott Fink, Jennifer Hogan

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/US_Buyers_Lanterns_and_Jewellery.xlsx
+++ b/US_Buyers_Lanterns_and_Jewellery.xlsx
@@ -504,9 +504,9 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -520,7 +520,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared: 22 October 2026  |  10 buyers: 5 Lanterns, 5 Jewellery</t>
+          <t>Prepared: 23 October 2026  |  10 buyers: 5 Lanterns, 5 Jewellery  |  US Customs import records, re-verified today</t>
         </is>
       </c>
     </row>
@@ -573,27 +573,27 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Buying Desk - Seasonal &amp; Home</t>
+          <t>Buying Desk - Seasonal &amp; Home Decor</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Costco Wholesale Corporation</t>
+          <t>World Market (Cost Plus World Market)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Issaquah, WA</t>
+          <t>Alameda, CA</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>https://www.costco.com</t>
+          <t>https://www.worldmarket.com</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Vendor submissions via Costco Supplier/Vendor Inquiry on costco.com</t>
+          <t>1201 Marina Village Pkwy, Alameda, CA 94501 | vendor enquiries via worldmarket.com</t>
         </is>
       </c>
     </row>
@@ -608,27 +608,27 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Buying Desk - Home &amp; Seasonal Decor</t>
+          <t>Buying Desk - Seasonal / Outdoor Decor</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Fred Meyer (The Kroger Co.)</t>
+          <t>Lowe's Companies, Inc. (L G Sourcing Inc.)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Wilkesboro, NC</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>https://www.fredmeyer.com</t>
+          <t>https://www.lowes.com</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Vendor/partner enquiries via fredmeyer.com; buying office Portland, OR</t>
+          <t>1605 Curtis Bridge Rd, Wilkesboro, NC 28697 | supplier onboarding via lowes.com</t>
         </is>
       </c>
     </row>
@@ -643,31 +643,31 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Cindy Kretzinger - Head of Product Development &amp; Merchandising</t>
+          <t>Buying Desk - Seasonal Home Decor</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Pier 1 Imports (Omni Retail Enterprises)</t>
+          <t>Family Dollar Stores, Inc.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Fort Worth, TX</t>
+          <t>Chesapeake, VA</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>https://www.pier1.com</t>
+          <t>https://www.familydollar.com</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Product development &amp; merchandising desk via pier1.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="49" customHeight="1">
+          <t>500 Volvo Pkwy, Chesapeake, VA 23320 | supplier onboarding via familydollar.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
@@ -678,27 +678,27 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Ashok 'Ash' Pamani - President / Owner (imports: Mahinder Pamani, Imports Manager)</t>
+          <t>Pat Dolan - Owner (A-Boy Supply Co. dba Globe Lighting)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Style Asia Inc.</t>
+          <t>Globe Lighting (A-Boy Supply Co.)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Moonachie, NJ</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>https://styleasia.net</t>
+          <t>https://www.globelighting.com</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>contact@styleasia.net | +1 (201) 460-9611 | toll-free (800) 522-7465</t>
+          <t>+1 (503) 225-9009 | +1 (800) 689-1000</t>
         </is>
       </c>
     </row>
@@ -713,31 +713,31 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Buying Desk - Hardlines / General Merchandise</t>
+          <t>Cindy Kretzinger - Head of Product Development &amp; Merchandising</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Kmart Corporation (Transformco)</t>
+          <t>Pier 1 Imports (Omni Retail Enterprises)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Hoffman Estates, IL</t>
+          <t>Fort Worth, TX</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>https://www.kmart.com</t>
+          <t>https://www.pier1.com</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Vendor enquiries via kmart.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
+          <t>100 Pier 1 Place, Fort Worth, TX 76102 | product development desk via pier1.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="19" customHeight="1">
       <c r="A10" s="7" t="n">
         <v>6</v>
       </c>
@@ -748,27 +748,27 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Buying Desk - Fashion Jewellery &amp; Accessories</t>
+          <t>Gavin Marks - Principal / Owner</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>The Avon Company (Avon Products, Inc.)</t>
+          <t>DM Merchandising, Inc.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Elmhurst, IL</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>https://www.avon.com</t>
+          <t>https://247dm.com</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Merchandising via avon.com; office 165 Broadway, New York, NY 10006</t>
+          <t>+1 (630) 782-2700 | +1 (800) 548-6784</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>scott@barryowen.com | orders@barryowen.com | +1 (323) 724-4800</t>
+          <t>scott@barryowen.com | +1 (323) 724-4800 | (800) 682-6682</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
+    <row r="13" ht="49" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
@@ -858,26 +858,26 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Dollar General Corporation</t>
+          <t>Big Lots (Variety Wholesalers, Inc.)</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Goodlettsville, TN</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>https://www.dollargeneral.com</t>
+          <t>https://www.biglots.com</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Supplier onboarding via Dollar General supplier portal / vendor enquiry</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="19" customHeight="1">
+          <t>200 E. Campus View Blvd, Suite 310, Columbus, OH 43235 | vendor enquiries via biglots.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="7" t="n">
         <v>10</v>
       </c>
@@ -893,12 +893,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Eastern Nationwide Supply Inc.</t>
+          <t>5 And 2 Co., Inc.</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Commerce, CA</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>1261 Broadway, Suite 701, New York, NY 10001</t>
+          <t>+1 (323) 728-2255 | 2727 Supply Ave, Commerce, CA 90040</t>
         </is>
       </c>
     </row>
@@ -944,14 +944,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1016,13 +1016,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="49" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Costco Wholesale Corporation</t>
+          <t>World Market (Cost Plus World Market)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1032,42 +1032,42 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>999 Lake Drive, Issaquah, WA 98027</t>
+          <t>1201 Marina Village Pkwy, Alameda, CA 94501</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Large solar base lantern (803 cartons)</t>
+          <t>Paraffin candles and woodenware (1,877 cartons, PO 200323279 / 200330503)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>China - Yantian</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Elizabeth, NJ</t>
+          <t>Oakland, CA</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Medium - solar / garden decor lanterns</t>
+          <t>High - imported home decor, lanterns and candle accessories are core lines</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Active - membership warehouse club; new vendors via Costco vendor programme</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
+          <t>Active - ~250 stores, privately held (Kingswood Capital Management)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="49" customHeight="1">
       <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Fred Meyer (The Kroger Co.)</t>
+          <t>Lowe's Companies, Inc. (L G Sourcing Inc.)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -1077,42 +1077,42 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>3800 SE 22nd Ave, Portland, OR 97202</t>
+          <t>Lowe's sourcing: 1605 Curtis Bridge Rd, Wilkesboro, NC 28697 (HQ: Mooresville, NC)</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Resin birdfeeder, straw bird house, lantern</t>
+          <t>Outdoor decor, lighted yard pieces, trees and wreaths</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>South Korea - Busan</t>
+          <t>China - Yantian</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Savannah, GA</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Medium-High - seasonal home decor</t>
+          <t>Medium-High - solar and decorative outdoor lanterns for seasonal sets</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>Active - Kroger banner, ~130 stores in the Pacific Northwest</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
+          <t>Active - Fortune 50 home-improvement retailer, 1,700+ stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="49" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Pier 1 Imports (Omni Retail Enterprises)</t>
+          <t>Family Dollar Stores, Inc.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1122,42 +1122,42 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>100 Pier 1 Place, Fort Worth, TX 76102</t>
+          <t>500 Volvo Pkwy, Chesapeake, VA 23320 (import DC on record: 10401 Old Monroe Rd, Matthews, NC)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Metal lanterns (44 cartons), with candle holders and other decor</t>
+          <t>Candle holders and Halloween / seasonal decor assortment</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>China - Ningbo</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Long Beach, CA</t>
+          <t>Portsmouth, VA</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>High - decorative metal lanterns</t>
+          <t>Medium - value-priced seasonal decor and candle lanterns</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Active - online-only since 2020; sourcing led by Omni Retail Enterprises</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="49" customHeight="1">
+          <t>Active - ~7,100 stores; standalone since 2025 (Brigade / Macellum / Arkhouse)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Style Asia Inc.</t>
+          <t>Globe Lighting (A-Boy Supply Co.)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1167,32 +1167,32 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>101 Moonachie Avenue, Moonachie, NJ 07074</t>
+          <t>1919 NW 19th Ave, Portland, OR 97209</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Lantern, steel flask, plastic container, pen</t>
+          <t>Lighting fixtures - brass table, desk and floor lamps (178 cartons)</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>China - Ningbo</t>
+          <t>China - Yantian</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>High - vintage LED lanterns in current catalogue; direct importer</t>
+          <t>High - lighting retailer/importer; buys decorative lamps and lanterns</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Active - importer &amp; wholesale distributor since 1985 (best-fit wholesale lead)</t>
+          <t>Active - 14 stores across OR / WA / ID under Globe Lighting &amp; Seattle Lighting</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Kmart Corporation (Transformco)</t>
+          <t>Pier 1 Imports (Omni Retail Enterprises)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1212,32 +1212,32 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>3333 Beverly Road, Hoffman Estates, IL 60179</t>
+          <t>100 Pier 1 Place, Fort Worth, TX 76102</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Rechargeable 3-in-1 lantern</t>
+          <t>Metal lanterns (44 cartons) with candle holders and decor</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Long Beach, CA</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Low-Medium - utility / camping lanterns rather than decorative</t>
+          <t>High - decorative metal lanterns are a signature Pier 1 category</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Limited - few stores remain under Transformco; kmart.com still trading</t>
+          <t>Active - online-first brand owned by Omni Retail Enterprises</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>The Avon Company (Avon Products, Inc.)</t>
+          <t>DM Merchandising, Inc.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -1257,17 +1257,17 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>165 Broadway, New York, NY 10006</t>
+          <t>835 N Church Ct, Elmhurst, IL 60126</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Jewelry - P.O. 69175211 / 69175212 / 69175813</t>
+          <t>Metal keychains, rings and necklaces; festival jewellery accessories</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1277,12 +1277,12 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>High - fashion jewellery is a core Avon category (Beauty Plus)</t>
+          <t>High - fashion jewellery and accessories are a core DM category</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Active - US business operates as The Avon Company</t>
+          <t>Active - 50+ years in gifts/accessories, 3,000+ SKUs, 20+ in-house brands</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Imitation jewelry (lead &amp; nickel free); pendant bracelets</t>
+          <t>Imitation jewellery (lead &amp; nickel free) and pendant bracelets</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1322,12 +1322,12 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>High - costume jewellery importer-wholesaler (also Barry-Owen Gift &amp; Home)</t>
+          <t>High - costume-jewellery importer-wholesaler, also runs Barry-Owen Gift &amp; Home</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Active - fresh imitation-jewellery imports recorded in 2026</t>
+          <t>Active - fresh imitation-jewellery imports recorded through 2026</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Travel jewelry, luggage tag, PVC bag, business-card case, passport cover</t>
+          <t>Travel jewellery cases, charms and gift accessories</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Medium - travel jewellery &amp; gift accessories (wholesale to 4,000+ stores)</t>
+          <t>Medium - travel jewellery and gift accessories, wholesale to 4,000+ stores</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Dollar General Corporation</t>
+          <t>Big Lots (Variety Wholesalers, Inc.)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1392,42 +1392,42 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>100 Mission Ridge, Goodlettsville, TN 37072</t>
+          <t>200 E. Campus View Blvd, Suite 310, Columbus, OH 43235</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>'Fairy N Jewel' necklace</t>
+          <t>Fashion jewellery sets - bracelets, necklaces, rings, earrings, tiaras</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>China - Yantian</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Portsmouth, VA</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>High - high-volume fashion jewellery and accessories</t>
+          <t>High - impulse fashion jewellery and accessory sets</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Active - ~20,000 stores; central buying from Goodlettsville</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="49" customHeight="1">
+          <t>Active - 217 stores; bought out of bankruptcy by Variety Wholesalers (2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="7" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Eastern Nationwide Supply Inc.</t>
+          <t>5 And 2 Co., Inc.</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>1261 Broadway, Suite 701, New York, NY 10001</t>
+          <t>2727 Supply Ave, Commerce, CA 90040</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Bangles, earrings, choker necklace and tie sets</t>
+          <t>Bracelet, necklace and earring sets (296 cartons)</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -1452,17 +1452,17 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>San Pedro, CA</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>High - pure-play fashion-jewellery importer in the NYC jewellery district</t>
+          <t>High - pure-play fashion-jewellery importer in the LA wholesale district</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Active - jewellery-set imports recorded through 2026</t>
+          <t>Active - importer / wholesale showroom; approach by phone or in person</t>
         </is>
       </c>
     </row>

</xml_diff>